<commit_message>
Deep dive analysis in bikes model and colour
</commit_message>
<xml_diff>
--- a/Project-5-AdventureWorks-Sales-Performance-Analysis/excel/02_deep_dive/02_root_cause_analysis.xlsx
+++ b/Project-5-AdventureWorks-Sales-Performance-Analysis/excel/02_deep_dive/02_root_cause_analysis.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="bikes_subcategory" sheetId="1" state="visible" r:id="rId3"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="35">
   <si>
     <t xml:space="preserve">modelname</t>
   </si>
@@ -129,9 +129,6 @@
     <t xml:space="preserve">Sum - qty</t>
   </si>
   <si>
-    <t xml:space="preserve">Delta_Profit</t>
-  </si>
-  <si>
     <t xml:space="preserve">Profit_Delta</t>
   </si>
 </sst>
@@ -144,11 +141,12 @@
     <numFmt numFmtId="165" formatCode="0"/>
     <numFmt numFmtId="166" formatCode="0.00"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -170,10 +168,18 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -198,7 +204,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="23">
+  <borders count="31">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -214,10 +220,38 @@
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
+      <left style="medium"/>
+      <right style="thin"/>
+      <top style="medium"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
       <left style="thin"/>
       <right style="thin"/>
       <top style="medium"/>
       <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top style="medium"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="medium"/>
+      <top style="medium"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="medium"/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
@@ -235,6 +269,13 @@
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="medium"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
       <left style="medium"/>
       <right style="thin"/>
       <top style="thin"/>
@@ -242,14 +283,21 @@
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
-      <left/>
-      <right style="medium"/>
+      <left style="thin"/>
+      <right style="thin"/>
       <top style="thin"/>
-      <bottom style="thin"/>
+      <bottom/>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin"/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
       <right style="thin"/>
       <top style="thin"/>
       <bottom/>
@@ -264,6 +312,34 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
       <right style="thin"/>
       <top/>
       <bottom style="thin"/>
@@ -291,13 +367,6 @@
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right/>
-      <top/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right style="medium"/>
       <top/>
@@ -307,13 +376,6 @@
     <border diagonalUp="false" diagonalDown="false">
       <left style="medium"/>
       <right style="thin"/>
-      <top style="thin"/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right/>
       <top style="thin"/>
       <bottom/>
       <diagonal/>
@@ -333,31 +395,31 @@
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
-      <left/>
+      <left style="medium"/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="medium"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="medium"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
       <right/>
-      <top style="thin"/>
-      <bottom/>
+      <top/>
+      <bottom style="medium"/>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left/>
-      <right/>
+      <right style="medium"/>
       <top/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left/>
-      <right style="thin"/>
-      <top/>
-      <bottom style="thin"/>
+      <bottom style="medium"/>
       <diagonal/>
     </border>
   </borders>
@@ -385,24 +447,50 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="54">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -410,47 +498,51 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="22" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="22" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="7" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="22" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="22" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -458,159 +550,139 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="7" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="7" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="12" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="13" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="8" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="15" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="16" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="16" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="9" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="18" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="19" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="20" xfId="21" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="21" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="22" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="18" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="23" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="24" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="25" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="26" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="23" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="23" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="25" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="13" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="14" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="7" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="9" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="27" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="16" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="17" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="18" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="28" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="13" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="14" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="3" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="6" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="16" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="19" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="19" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="20" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="21" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="21" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="22" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="29" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="30" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -622,15 +694,15 @@
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="Pivot Table Corner" xfId="20"/>
-    <cellStyle name="Pivot Table Value" xfId="21"/>
+    <cellStyle name="Pivot Table Category" xfId="20"/>
+    <cellStyle name="Pivot Table Corner" xfId="21"/>
     <cellStyle name="Pivot Table Field" xfId="22"/>
-    <cellStyle name="Pivot Table Category" xfId="23"/>
+    <cellStyle name="Pivot Table Result" xfId="23"/>
     <cellStyle name="Pivot Table Title" xfId="24"/>
-    <cellStyle name="Pivot Table Result" xfId="25"/>
+    <cellStyle name="Pivot Table Value" xfId="25"/>
     <cellStyle name="Yellow" xfId="26"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="6">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -664,6 +736,9 @@
     </dxf>
     <dxf>
       <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="2"/>
         <color rgb="FFCC0000"/>
       </font>
       <fill>
@@ -674,17 +749,17 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </dxf>
     <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="2"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="General"/>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </dxf>
   </dxfs>
   <colors>
@@ -769,8 +844,12 @@
             </a:pPr>
             <a:r>
               <a:rPr sz="1400" b="1" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>Profit Delta per Product Bikes (2021→2022)</a:t>
             </a:r>
@@ -800,7 +879,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Delta_Profit</c:v>
+                  <c:v>Profit_Delta</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -850,6 +929,30 @@
               </a:ln>
             </c:spPr>
           </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:invertIfNegative val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="00a933"/>
+              </a:solidFill>
+              <a:ln w="0">
+                <a:noFill/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="10"/>
+            <c:invertIfNegative val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="00a933"/>
+              </a:solidFill>
+              <a:ln w="0">
+                <a:noFill/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
           <c:dLbls>
             <c:dLbl>
               <c:idx val="0"/>
@@ -865,6 +968,7 @@
                       </a:solidFill>
                       <a:uFillTx/>
                       <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
@@ -891,6 +995,7 @@
                       </a:solidFill>
                       <a:uFillTx/>
                       <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
@@ -917,6 +1022,59 @@
                       </a:solidFill>
                       <a:uFillTx/>
                       <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
+                    </a:defRPr>
+                  </a:pPr>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:separator> </c:separator>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:numFmt formatCode="General" sourceLinked="1"/>
+              <c:txPr>
+                <a:bodyPr wrap="none"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
+                      <a:uFillTx/>
+                      <a:latin typeface="Arial"/>
+                    </a:defRPr>
+                  </a:pPr>
+                </a:p>
+              </c:txPr>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:separator> </c:separator>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="10"/>
+              <c:numFmt formatCode="General" sourceLinked="1"/>
+              <c:txPr>
+                <a:bodyPr wrap="none"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
+                      <a:uFillTx/>
+                      <a:latin typeface="Arial"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
@@ -936,8 +1094,12 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
+                    <a:ea typeface="DejaVu Sans"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
@@ -1028,28 +1190,28 @@
                   <c:v>-95221.9827</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-4737.45959999983</c:v>
+                  <c:v>-4737.4596</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-199.067999999999</c:v>
+                  <c:v>-199.068000000001</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2403.84000000003</c:v>
+                  <c:v>2403.84</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>19767.0656000001</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>22284.6269</c:v>
+                  <c:v>22284.6268999999</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>28652.3304000001</c:v>
+                  <c:v>28652.3304000002</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>44413.3731999994</c:v>
+                  <c:v>44413.3731999989</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>45158.2919999979</c:v>
+                  <c:v>45158.291999998</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>178740.719999998</c:v>
@@ -1063,17 +1225,17 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="0"/>
-        <c:axId val="94428738"/>
-        <c:axId val="51239736"/>
+        <c:axId val="57382395"/>
+        <c:axId val="1649432"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="94428738"/>
+        <c:axId val="57382395"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1090,13 +1252,17 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="51239736"/>
+        <c:crossAx val="1649432"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1104,7 +1270,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="51239736"/>
+        <c:axId val="1649432"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1119,7 +1285,7 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1136,13 +1302,17 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94428738"/>
+        <c:crossAx val="57382395"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1170,8 +1340,12 @@
         <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
               <a:uFillTx/>
               <a:latin typeface="Arial"/>
+              <a:ea typeface="DejaVu Sans"/>
             </a:defRPr>
           </a:pPr>
         </a:p>
@@ -1196,15 +1370,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>65880</xdr:colOff>
+      <xdr:colOff>46440</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>7560</xdr:rowOff>
+      <xdr:rowOff>26640</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>432000</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>158760</xdr:rowOff>
+      <xdr:colOff>412200</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>14760</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1212,8 +1386,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="5574600" y="495360"/>
-        <a:ext cx="5759640" cy="3239640"/>
+        <a:off x="5556240" y="514440"/>
+        <a:ext cx="5760360" cy="3239280"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2209,1084 +2383,1084 @@
   <dimension ref="A1:I37"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="11.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="5.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="4.07"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="7" style="2" width="16.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="11.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="20.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="5.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="4.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="7" style="3" width="16.74"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="1" t="n">
+      <c r="D2" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="E2" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="F2" s="2" t="n">
         <v>572</v>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="G2" s="3" t="n">
         <v>1247853.75</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="3" t="n">
         <v>755431.1336</v>
       </c>
-      <c r="I2" s="2" t="n">
+      <c r="I2" s="3" t="n">
         <v>492422.616400001</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="1" t="n">
+      <c r="D3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E3" s="1" t="n">
+      <c r="E3" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="F3" s="1" t="n">
+      <c r="F3" s="2" t="n">
         <v>847</v>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="G3" s="3" t="n">
         <v>1735586.17539997</v>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="3" t="n">
         <v>936621.07000002</v>
       </c>
-      <c r="I3" s="2" t="n">
+      <c r="I3" s="3" t="n">
         <v>798965.10539999</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="1" t="n">
+      <c r="D4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E4" s="1" t="n">
+      <c r="E4" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="F4" s="1" t="n">
+      <c r="F4" s="2" t="n">
         <v>101</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="G4" s="3" t="n">
         <v>74977.35</v>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="3" t="n">
         <v>46605.9248</v>
       </c>
-      <c r="I4" s="2" t="n">
+      <c r="I4" s="3" t="n">
         <v>28371.4252</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="1" t="n">
+      <c r="D5" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="1" t="n">
+      <c r="E5" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="F5" s="1" t="n">
+      <c r="F5" s="2" t="n">
         <v>613</v>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="G5" s="3" t="n">
         <v>613268.1875</v>
       </c>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="3" t="n">
         <v>371262.9596</v>
       </c>
-      <c r="I5" s="2" t="n">
+      <c r="I5" s="3" t="n">
         <v>242005.227899996</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="1" t="n">
+      <c r="D6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="1" t="n">
+      <c r="E6" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="F6" s="1" t="n">
+      <c r="F6" s="2" t="n">
         <v>809</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="G6" s="3" t="n">
         <v>1675778.45639998</v>
       </c>
-      <c r="H6" s="2" t="n">
+      <c r="H6" s="3" t="n">
         <v>904345.423099993</v>
       </c>
-      <c r="I6" s="2" t="n">
+      <c r="I6" s="3" t="n">
         <v>771433.033300014</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="1" t="n">
+      <c r="D7" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E7" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="F7" s="1" t="n">
+      <c r="F7" s="2" t="n">
         <v>323</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G7" s="3" t="n">
         <v>754122.524999998</v>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="H7" s="3" t="n">
         <v>464022.2588</v>
       </c>
-      <c r="I7" s="2" t="n">
+      <c r="I7" s="3" t="n">
         <v>290100.266199999</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="1" t="n">
+      <c r="D8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="E8" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="F8" s="1" t="n">
+      <c r="F8" s="2" t="n">
         <v>596</v>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="G8" s="3" t="n">
         <v>321834.039999997</v>
       </c>
-      <c r="H8" s="2" t="n">
+      <c r="H8" s="3" t="n">
         <v>204815.161600001</v>
       </c>
-      <c r="I8" s="2" t="n">
+      <c r="I8" s="3" t="n">
         <v>117018.8784</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="1" t="n">
+      <c r="D9" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="1" t="n">
+      <c r="E9" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="F9" s="1" t="n">
+      <c r="F9" s="2" t="n">
         <v>159</v>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="G9" s="3" t="n">
         <v>193161.150000001</v>
       </c>
-      <c r="H9" s="2" t="n">
+      <c r="H9" s="3" t="n">
         <v>120068.9772</v>
       </c>
-      <c r="I9" s="2" t="n">
+      <c r="I9" s="3" t="n">
         <v>73092.1728000002</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="1" t="n">
+      <c r="D10" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="1" t="n">
+      <c r="E10" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="F10" s="1" t="n">
+      <c r="F10" s="2" t="n">
         <v>224</v>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="G10" s="3" t="n">
         <v>534031.680000001</v>
       </c>
-      <c r="H10" s="2" t="n">
+      <c r="H10" s="3" t="n">
         <v>331954.0896</v>
       </c>
-      <c r="I10" s="2" t="n">
+      <c r="I10" s="3" t="n">
         <v>202077.590399999</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="1" t="n">
+      <c r="D11" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E11" s="1" t="n">
+      <c r="E11" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="F11" s="1" t="n">
+      <c r="F11" s="2" t="n">
         <v>163</v>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="G11" s="3" t="n">
         <v>113953.0066</v>
       </c>
-      <c r="H11" s="2" t="n">
+      <c r="H11" s="3" t="n">
         <v>67342.8469</v>
       </c>
-      <c r="I11" s="2" t="n">
+      <c r="I11" s="3" t="n">
         <v>46610.1597</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D12" s="1" t="n">
+      <c r="D12" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="1" t="n">
+      <c r="E12" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="F12" s="1" t="n">
+      <c r="F12" s="2" t="n">
         <v>203</v>
       </c>
-      <c r="G12" s="2" t="n">
+      <c r="G12" s="3" t="n">
         <v>156206.47</v>
       </c>
-      <c r="H12" s="2" t="n">
+      <c r="H12" s="3" t="n">
         <v>85215.0152</v>
       </c>
-      <c r="I12" s="2" t="n">
+      <c r="I12" s="3" t="n">
         <v>70991.4548000001</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D13" s="1" t="n">
+      <c r="D13" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="1" t="n">
+      <c r="E13" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="F13" s="1" t="n">
+      <c r="F13" s="2" t="n">
         <v>93</v>
       </c>
-      <c r="G13" s="2" t="n">
+      <c r="G13" s="3" t="n">
         <v>52544.07</v>
       </c>
-      <c r="H13" s="2" t="n">
+      <c r="H13" s="3" t="n">
         <v>28664.2647</v>
       </c>
-      <c r="I13" s="2" t="n">
+      <c r="I13" s="3" t="n">
         <v>23879.8053</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D14" s="1" t="n">
+      <c r="D14" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="1" t="n">
+      <c r="E14" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="F14" s="1" t="n">
+      <c r="F14" s="2" t="n">
         <v>214</v>
       </c>
-      <c r="G14" s="2" t="n">
+      <c r="G14" s="3" t="n">
         <v>510190.980000001</v>
       </c>
-      <c r="H14" s="2" t="n">
+      <c r="H14" s="3" t="n">
         <v>317134.7106</v>
       </c>
-      <c r="I14" s="2" t="n">
+      <c r="I14" s="3" t="n">
         <v>193056.269399999</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D15" s="1" t="n">
+      <c r="D15" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E15" s="1" t="n">
+      <c r="E15" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="F15" s="1" t="n">
+      <c r="F15" s="2" t="n">
         <v>170</v>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="G15" s="3" t="n">
         <v>118846.694</v>
       </c>
-      <c r="H15" s="2" t="n">
+      <c r="H15" s="3" t="n">
         <v>70234.871</v>
       </c>
-      <c r="I15" s="2" t="n">
+      <c r="I15" s="3" t="n">
         <v>48611.823</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C16" s="0" t="n">
+      <c r="C16" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D16" s="1" t="n">
+      <c r="D16" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="E16" s="1" t="n">
+      <c r="E16" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="F16" s="1" t="n">
+      <c r="F16" s="2" t="n">
         <v>118</v>
       </c>
-      <c r="G16" s="2" t="n">
+      <c r="G16" s="3" t="n">
         <v>18762</v>
       </c>
-      <c r="H16" s="2" t="n">
+      <c r="H16" s="3" t="n">
         <v>7016.98800000001</v>
       </c>
-      <c r="I16" s="2" t="n">
+      <c r="I16" s="3" t="n">
         <v>11745.012</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="C17" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D17" s="1" t="n">
+      <c r="D17" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E17" s="1" t="n">
+      <c r="E17" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="F17" s="1" t="n">
+      <c r="F17" s="2" t="n">
         <v>311</v>
       </c>
-      <c r="G17" s="2" t="n">
+      <c r="G17" s="3" t="n">
         <v>529007.889999998</v>
       </c>
-      <c r="H17" s="2" t="n">
+      <c r="H17" s="3" t="n">
         <v>336660.610000001</v>
       </c>
-      <c r="I17" s="2" t="n">
+      <c r="I17" s="3" t="n">
         <v>192347.280000001</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="0" t="s">
+      <c r="C18" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D18" s="1" t="n">
+      <c r="D18" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E18" s="1" t="n">
+      <c r="E18" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="F18" s="1" t="n">
+      <c r="F18" s="2" t="n">
         <v>113</v>
       </c>
-      <c r="G18" s="2" t="n">
+      <c r="G18" s="3" t="n">
         <v>83885.5500000001</v>
       </c>
-      <c r="H18" s="2" t="n">
+      <c r="H18" s="3" t="n">
         <v>52143.2623999999</v>
       </c>
-      <c r="I18" s="2" t="n">
+      <c r="I18" s="3" t="n">
         <v>31742.2876</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C19" s="0" t="s">
+      <c r="C19" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D19" s="1" t="n">
+      <c r="D19" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E19" s="1" t="n">
+      <c r="E19" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="F19" s="1" t="n">
+      <c r="F19" s="2" t="n">
         <v>99</v>
       </c>
-      <c r="G19" s="2" t="n">
+      <c r="G19" s="3" t="n">
         <v>53459.01</v>
       </c>
-      <c r="H19" s="2" t="n">
+      <c r="H19" s="3" t="n">
         <v>29163.3902999999</v>
       </c>
-      <c r="I19" s="2" t="n">
+      <c r="I19" s="3" t="n">
         <v>24295.6197</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C20" s="0" t="n">
+      <c r="C20" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D20" s="1" t="n">
+      <c r="D20" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="E20" s="1" t="n">
+      <c r="E20" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="F20" s="1" t="n">
+      <c r="F20" s="2" t="n">
         <v>135</v>
       </c>
-      <c r="G20" s="2" t="n">
+      <c r="G20" s="3" t="n">
         <v>16200</v>
       </c>
-      <c r="H20" s="2" t="n">
+      <c r="H20" s="3" t="n">
         <v>6058.80000000001</v>
       </c>
-      <c r="I20" s="2" t="n">
+      <c r="I20" s="3" t="n">
         <v>10141.2</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="C21" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D21" s="1" t="n">
+      <c r="D21" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E21" s="1" t="n">
+      <c r="E21" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="F21" s="1" t="n">
+      <c r="F21" s="2" t="n">
         <v>234</v>
       </c>
-      <c r="G21" s="2" t="n">
+      <c r="G21" s="3" t="n">
         <v>510485.625</v>
       </c>
-      <c r="H21" s="2" t="n">
+      <c r="H21" s="3" t="n">
         <v>309040.0092</v>
       </c>
-      <c r="I21" s="2" t="n">
+      <c r="I21" s="3" t="n">
         <v>201445.6158</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="B22" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C22" s="0" t="s">
+      <c r="C22" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D22" s="1" t="n">
+      <c r="D22" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E22" s="1" t="n">
+      <c r="E22" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="F22" s="1" t="n">
+      <c r="F22" s="2" t="n">
         <v>724</v>
       </c>
-      <c r="G22" s="2" t="n">
+      <c r="G22" s="3" t="n">
         <v>1483547.09679998</v>
       </c>
-      <c r="H22" s="2" t="n">
+      <c r="H22" s="3" t="n">
         <v>800606.440000013</v>
       </c>
-      <c r="I22" s="2" t="n">
+      <c r="I22" s="3" t="n">
         <v>682940.656799996</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C23" s="0" t="s">
+      <c r="C23" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D23" s="1" t="n">
+      <c r="D23" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E23" s="1" t="n">
+      <c r="E23" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="F23" s="1" t="n">
+      <c r="F23" s="2" t="n">
         <v>155</v>
       </c>
-      <c r="G23" s="2" t="n">
+      <c r="G23" s="3" t="n">
         <v>115064.25</v>
       </c>
-      <c r="H23" s="2" t="n">
+      <c r="H23" s="3" t="n">
         <v>71523.9439999998</v>
       </c>
-      <c r="I23" s="2" t="n">
+      <c r="I23" s="3" t="n">
         <v>43540.3060000001</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B24" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C24" s="0" t="s">
+      <c r="C24" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D24" s="1" t="n">
+      <c r="D24" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E24" s="1" t="n">
+      <c r="E24" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="F24" s="1" t="n">
+      <c r="F24" s="2" t="n">
         <v>132</v>
       </c>
-      <c r="G24" s="2" t="n">
+      <c r="G24" s="3" t="n">
         <v>74578.68</v>
       </c>
-      <c r="H24" s="2" t="n">
+      <c r="H24" s="3" t="n">
         <v>40684.7628000001</v>
       </c>
-      <c r="I24" s="2" t="n">
+      <c r="I24" s="3" t="n">
         <v>33893.9171999999</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+      <c r="A25" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="B25" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C25" s="0" t="s">
+      <c r="C25" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D25" s="1" t="n">
+      <c r="D25" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E25" s="1" t="n">
+      <c r="E25" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="F25" s="1" t="n">
+      <c r="F25" s="2" t="n">
         <v>391</v>
       </c>
-      <c r="G25" s="2" t="n">
+      <c r="G25" s="3" t="n">
         <v>932171.369999993</v>
       </c>
-      <c r="H25" s="2" t="n">
+      <c r="H25" s="3" t="n">
         <v>579437.718900003</v>
       </c>
-      <c r="I25" s="2" t="n">
+      <c r="I25" s="3" t="n">
         <v>352733.651099997</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+      <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="0" t="s">
+      <c r="B26" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="0" t="s">
+      <c r="C26" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D26" s="1" t="n">
+      <c r="D26" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E26" s="1" t="n">
+      <c r="E26" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="F26" s="1" t="n">
+      <c r="F26" s="2" t="n">
         <v>330</v>
       </c>
-      <c r="G26" s="2" t="n">
+      <c r="G26" s="3" t="n">
         <v>253931.699999999</v>
       </c>
-      <c r="H26" s="2" t="n">
+      <c r="H26" s="3" t="n">
         <v>138526.872</v>
       </c>
-      <c r="I26" s="2" t="n">
+      <c r="I26" s="3" t="n">
         <v>115404.827999999</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+      <c r="A27" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="0" t="s">
+      <c r="B27" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C27" s="0" t="s">
+      <c r="C27" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D27" s="1" t="n">
+      <c r="D27" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E27" s="1" t="n">
+      <c r="E27" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="F27" s="1" t="n">
+      <c r="F27" s="2" t="n">
         <v>600</v>
       </c>
-      <c r="G27" s="2" t="n">
+      <c r="G27" s="3" t="n">
         <v>1020594</v>
       </c>
-      <c r="H27" s="2" t="n">
+      <c r="H27" s="3" t="n">
         <v>649506.000000004</v>
       </c>
-      <c r="I27" s="2" t="n">
+      <c r="I27" s="3" t="n">
         <v>371087.999999999</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
+      <c r="A28" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B28" s="0" t="s">
+      <c r="B28" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="0" t="n">
+      <c r="C28" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D28" s="1" t="n">
+      <c r="D28" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="E28" s="1" t="n">
+      <c r="E28" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="F28" s="1" t="n">
+      <c r="F28" s="2" t="n">
         <v>167</v>
       </c>
-      <c r="G28" s="2" t="n">
+      <c r="G28" s="3" t="n">
         <v>20040</v>
       </c>
-      <c r="H28" s="2" t="n">
+      <c r="H28" s="3" t="n">
         <v>7494.96000000002</v>
       </c>
-      <c r="I28" s="2" t="n">
+      <c r="I28" s="3" t="n">
         <v>12545.04</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
+      <c r="A29" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B29" s="0" t="s">
+      <c r="B29" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C29" s="0" t="s">
+      <c r="C29" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D29" s="1" t="n">
+      <c r="D29" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E29" s="1" t="n">
+      <c r="E29" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="F29" s="1" t="n">
+      <c r="F29" s="2" t="n">
         <v>161</v>
       </c>
-      <c r="G29" s="2" t="n">
+      <c r="G29" s="3" t="n">
         <v>119518.35</v>
       </c>
-      <c r="H29" s="2" t="n">
+      <c r="H29" s="3" t="n">
         <v>74292.6127999998</v>
       </c>
-      <c r="I29" s="2" t="n">
+      <c r="I29" s="3" t="n">
         <v>45225.7372000001</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
+      <c r="A30" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B30" s="0" t="s">
+      <c r="B30" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C30" s="0" t="s">
+      <c r="C30" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D30" s="1" t="n">
+      <c r="D30" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E30" s="1" t="n">
+      <c r="E30" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="F30" s="1" t="n">
+      <c r="F30" s="2" t="n">
         <v>149</v>
       </c>
-      <c r="G30" s="2" t="n">
+      <c r="G30" s="3" t="n">
         <v>80458.5100000001</v>
       </c>
-      <c r="H30" s="2" t="n">
+      <c r="H30" s="3" t="n">
         <v>43892.3753</v>
       </c>
-      <c r="I30" s="2" t="n">
+      <c r="I30" s="3" t="n">
         <v>36566.1347</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
+      <c r="A31" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B31" s="0" t="s">
+      <c r="B31" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C31" s="0" t="n">
+      <c r="C31" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D31" s="1" t="n">
+      <c r="D31" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="E31" s="1" t="n">
+      <c r="E31" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="F31" s="1" t="n">
+      <c r="F31" s="2" t="n">
         <v>116</v>
       </c>
-      <c r="G31" s="2" t="n">
+      <c r="G31" s="3" t="n">
         <v>18444</v>
       </c>
-      <c r="H31" s="2" t="n">
+      <c r="H31" s="3" t="n">
         <v>6898.05600000001</v>
       </c>
-      <c r="I31" s="2" t="n">
+      <c r="I31" s="3" t="n">
         <v>11545.944</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
+      <c r="A32" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B32" s="0" t="s">
+      <c r="B32" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C32" s="0" t="s">
+      <c r="C32" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D32" s="1" t="n">
+      <c r="D32" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E32" s="1" t="n">
+      <c r="E32" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="F32" s="1" t="n">
+      <c r="F32" s="2" t="n">
         <v>826</v>
       </c>
-      <c r="G32" s="2" t="n">
+      <c r="G32" s="3" t="n">
         <v>446031.739999995</v>
       </c>
-      <c r="H32" s="2" t="n">
+      <c r="H32" s="3" t="n">
         <v>283854.569600002</v>
       </c>
-      <c r="I32" s="2" t="n">
+      <c r="I32" s="3" t="n">
         <v>162177.170399998</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="s">
+      <c r="A33" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B33" s="0" t="s">
+      <c r="B33" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C33" s="0" t="s">
+      <c r="C33" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D33" s="1" t="n">
+      <c r="D33" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E33" s="1" t="n">
+      <c r="E33" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="F33" s="1" t="n">
+      <c r="F33" s="2" t="n">
         <v>717</v>
       </c>
-      <c r="G33" s="2" t="n">
+      <c r="G33" s="3" t="n">
         <v>1485207.85319999</v>
       </c>
-      <c r="H33" s="2" t="n">
+      <c r="H33" s="3" t="n">
         <v>801502.680299996</v>
       </c>
-      <c r="I33" s="2" t="n">
+      <c r="I33" s="3" t="n">
         <v>683705.172900009</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="s">
+      <c r="A34" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B34" s="0" t="s">
+      <c r="B34" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C34" s="0" t="s">
+      <c r="C34" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D34" s="1" t="n">
+      <c r="D34" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E34" s="1" t="n">
+      <c r="E34" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="F34" s="1" t="n">
+      <c r="F34" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="G34" s="2" t="n">
+      <c r="G34" s="3" t="n">
         <v>137438.4375</v>
       </c>
-      <c r="H34" s="2" t="n">
+      <c r="H34" s="3" t="n">
         <v>83203.0794</v>
       </c>
-      <c r="I34" s="2" t="n">
+      <c r="I34" s="3" t="n">
         <v>54235.3581</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
+      <c r="A35" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B35" s="0" t="s">
+      <c r="B35" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C35" s="0" t="s">
+      <c r="C35" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D35" s="1" t="n">
+      <c r="D35" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E35" s="1" t="n">
+      <c r="E35" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="F35" s="1" t="n">
+      <c r="F35" s="2" t="n">
         <v>202</v>
       </c>
-      <c r="G35" s="2" t="n">
+      <c r="G35" s="3" t="n">
         <v>245399.700000001</v>
       </c>
-      <c r="H35" s="2" t="n">
+      <c r="H35" s="3" t="n">
         <v>152540.4616</v>
       </c>
-      <c r="I35" s="2" t="n">
+      <c r="I35" s="3" t="n">
         <v>92859.2384000003</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="s">
+      <c r="A36" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B36" s="0" t="s">
+      <c r="B36" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C36" s="0" t="s">
+      <c r="C36" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D36" s="1" t="n">
+      <c r="D36" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E36" s="1" t="n">
+      <c r="E36" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="F36" s="1" t="n">
+      <c r="F36" s="2" t="n">
         <v>404</v>
       </c>
-      <c r="G36" s="2" t="n">
+      <c r="G36" s="3" t="n">
         <v>963164.279999992</v>
       </c>
-      <c r="H36" s="2" t="n">
+      <c r="H36" s="3" t="n">
         <v>598702.911600004</v>
       </c>
-      <c r="I36" s="2" t="n">
+      <c r="I36" s="3" t="n">
         <v>364461.368399997</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
+      <c r="A37" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B37" s="0" t="s">
+      <c r="B37" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C37" s="0" t="s">
+      <c r="C37" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D37" s="1" t="n">
+      <c r="D37" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E37" s="1" t="n">
+      <c r="E37" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="F37" s="1" t="n">
+      <c r="F37" s="2" t="n">
         <v>601</v>
       </c>
-      <c r="G37" s="2" t="n">
+      <c r="G37" s="3" t="n">
         <v>601262.9375</v>
       </c>
-      <c r="H37" s="2" t="n">
+      <c r="H37" s="3" t="n">
         <v>363995.169200001</v>
       </c>
-      <c r="I37" s="2" t="n">
+      <c r="I37" s="3" t="n">
         <v>237267.768299996</v>
       </c>
     </row>
@@ -3306,358 +3480,401 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="16.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="18.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="9.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="3" width="16.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="18.68"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>30</v>
       </c>
+      <c r="C1" s="0"/>
+      <c r="D1" s="0"/>
+      <c r="E1" s="0"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="0"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>30</v>
       </c>
+      <c r="C2" s="0"/>
+      <c r="D2" s="0"/>
+      <c r="E2" s="0"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="0"/>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0"/>
+      <c r="B3" s="0"/>
+      <c r="C3" s="0"/>
+      <c r="D3" s="0"/>
+      <c r="E3" s="0"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="0"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5"/>
-      <c r="B4" s="6" t="s">
+      <c r="A4" s="7"/>
+      <c r="B4" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="0"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5"/>
-      <c r="B5" s="7" t="n">
+      <c r="A5" s="11"/>
+      <c r="B5" s="12" t="n">
         <v>2021</v>
       </c>
-      <c r="C5" s="8"/>
-      <c r="D5" s="9" t="n">
+      <c r="C5" s="13"/>
+      <c r="D5" s="12" t="n">
         <v>2022</v>
       </c>
-      <c r="E5" s="9"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="0"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="19" t="s">
         <v>34</v>
       </c>
+      <c r="G6" s="0"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="16" t="n">
+      <c r="B7" s="21" t="n">
         <v>782522.8826</v>
       </c>
-      <c r="C7" s="17" t="n">
+      <c r="C7" s="22" t="n">
         <v>895</v>
       </c>
-      <c r="D7" s="16" t="n">
+      <c r="D7" s="21" t="n">
         <v>255680.9739</v>
       </c>
-      <c r="E7" s="17" t="n">
+      <c r="E7" s="22" t="n">
         <v>297</v>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="F7" s="23" t="n">
         <f aca="false">D7-B7</f>
         <v>-526841.9087</v>
       </c>
+      <c r="G7" s="0"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="20" t="n">
+      <c r="B8" s="25" t="n">
         <v>1570398.1387</v>
       </c>
-      <c r="C8" s="21" t="n">
+      <c r="C8" s="26" t="n">
         <v>1656</v>
       </c>
-      <c r="D8" s="20" t="n">
-        <v>1366645.8297</v>
-      </c>
-      <c r="E8" s="21" t="n">
+      <c r="D8" s="25" t="n">
+        <v>1366645.82970001</v>
+      </c>
+      <c r="E8" s="26" t="n">
         <v>1441</v>
       </c>
-      <c r="F8" s="22" t="n">
+      <c r="F8" s="27" t="n">
         <f aca="false">D8-B8</f>
         <v>-203752.308999999</v>
       </c>
+      <c r="G8" s="0"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="20" t="n">
+      <c r="B9" s="25" t="n">
         <v>95221.9827</v>
       </c>
-      <c r="C9" s="21" t="n">
+      <c r="C9" s="26" t="n">
         <v>333</v>
       </c>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="22" t="n">
+      <c r="D9" s="28"/>
+      <c r="E9" s="29"/>
+      <c r="F9" s="27" t="n">
         <f aca="false">D9-B9</f>
         <v>-95221.9827</v>
       </c>
+      <c r="G9" s="0"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="20" t="n">
+      <c r="B10" s="25" t="n">
         <v>242005.227899996</v>
       </c>
-      <c r="C10" s="21" t="n">
+      <c r="C10" s="26" t="n">
         <v>613</v>
       </c>
-      <c r="D10" s="20" t="n">
+      <c r="D10" s="25" t="n">
         <v>237267.768299996</v>
       </c>
-      <c r="E10" s="21" t="n">
+      <c r="E10" s="26" t="n">
         <v>601</v>
       </c>
-      <c r="F10" s="22" t="n">
+      <c r="F10" s="27" t="n">
         <f aca="false">D10-B10</f>
-        <v>-4737.45959999983</v>
-      </c>
+        <v>-4737.4596</v>
+      </c>
+      <c r="G10" s="0"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="20" t="n">
+      <c r="B11" s="25" t="n">
         <v>11745.012</v>
       </c>
-      <c r="C11" s="21" t="n">
+      <c r="C11" s="26" t="n">
         <v>118</v>
       </c>
-      <c r="D11" s="20" t="n">
+      <c r="D11" s="25" t="n">
         <v>11545.944</v>
       </c>
-      <c r="E11" s="21" t="n">
+      <c r="E11" s="26" t="n">
         <v>116</v>
       </c>
-      <c r="F11" s="22" t="n">
+      <c r="F11" s="27" t="n">
         <f aca="false">D11-B11</f>
-        <v>-199.067999999999</v>
-      </c>
+        <v>-199.068000000001</v>
+      </c>
+      <c r="G11" s="0"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="20" t="n">
+      <c r="B12" s="25" t="n">
         <v>10141.2</v>
       </c>
-      <c r="C12" s="21" t="n">
+      <c r="C12" s="26" t="n">
         <v>135</v>
       </c>
-      <c r="D12" s="20" t="n">
+      <c r="D12" s="25" t="n">
         <v>12545.04</v>
       </c>
-      <c r="E12" s="21" t="n">
+      <c r="E12" s="26" t="n">
         <v>167</v>
       </c>
-      <c r="F12" s="22" t="n">
+      <c r="F12" s="27" t="n">
         <f aca="false">D12-B12</f>
-        <v>2403.84000000003</v>
-      </c>
+        <v>2403.84</v>
+      </c>
+      <c r="G12" s="0"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="20" t="n">
+      <c r="B13" s="25" t="n">
         <v>73092.1728000002</v>
       </c>
-      <c r="C13" s="21" t="n">
+      <c r="C13" s="26" t="n">
         <v>159</v>
       </c>
-      <c r="D13" s="20" t="n">
+      <c r="D13" s="25" t="n">
         <v>92859.2384000003</v>
       </c>
-      <c r="E13" s="21" t="n">
+      <c r="E13" s="26" t="n">
         <v>202</v>
       </c>
-      <c r="F13" s="22" t="n">
+      <c r="F13" s="27" t="n">
         <f aca="false">D13-B13</f>
         <v>19767.0656000001</v>
       </c>
+      <c r="G13" s="0"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19" t="s">
+      <c r="A14" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="20" t="n">
-        <v>48175.4249999999</v>
-      </c>
-      <c r="C14" s="21" t="n">
+      <c r="B14" s="25" t="n">
+        <v>48175.425</v>
+      </c>
+      <c r="C14" s="26" t="n">
         <v>192</v>
       </c>
-      <c r="D14" s="20" t="n">
+      <c r="D14" s="25" t="n">
         <v>70460.0518999999</v>
       </c>
-      <c r="E14" s="21" t="n">
+      <c r="E14" s="26" t="n">
         <v>281</v>
       </c>
-      <c r="F14" s="22" t="n">
+      <c r="F14" s="27" t="n">
         <f aca="false">D14-B14</f>
-        <v>22284.6269</v>
-      </c>
+        <v>22284.6268999999</v>
+      </c>
+      <c r="G14" s="0"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="20" t="n">
-        <v>60113.7128000001</v>
-      </c>
-      <c r="C15" s="21" t="n">
+      <c r="B15" s="25" t="n">
+        <v>60113.7128</v>
+      </c>
+      <c r="C15" s="26" t="n">
         <v>214</v>
       </c>
-      <c r="D15" s="20" t="n">
+      <c r="D15" s="25" t="n">
         <v>88766.0432000002</v>
       </c>
-      <c r="E15" s="21" t="n">
+      <c r="E15" s="26" t="n">
         <v>316</v>
       </c>
-      <c r="F15" s="22" t="n">
+      <c r="F15" s="27" t="n">
         <f aca="false">D15-B15</f>
-        <v>28652.3304000001</v>
-      </c>
+        <v>28652.3304000002</v>
+      </c>
+      <c r="G15" s="0"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="19" t="s">
+      <c r="A16" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="20" t="n">
+      <c r="B16" s="25" t="n">
         <v>70991.4548000001</v>
       </c>
-      <c r="C16" s="21" t="n">
+      <c r="C16" s="26" t="n">
         <v>203</v>
       </c>
-      <c r="D16" s="20" t="n">
+      <c r="D16" s="25" t="n">
         <v>115404.827999999</v>
       </c>
-      <c r="E16" s="21" t="n">
+      <c r="E16" s="26" t="n">
         <v>330</v>
       </c>
-      <c r="F16" s="22" t="n">
+      <c r="F16" s="27" t="n">
         <f aca="false">D16-B16</f>
-        <v>44413.3731999994</v>
-      </c>
+        <v>44413.3731999989</v>
+      </c>
+      <c r="G16" s="0"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="19" t="s">
+      <c r="A17" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="20" t="n">
+      <c r="B17" s="25" t="n">
         <v>117018.8784</v>
       </c>
-      <c r="C17" s="21" t="n">
+      <c r="C17" s="26" t="n">
         <v>596</v>
       </c>
-      <c r="D17" s="20" t="n">
+      <c r="D17" s="25" t="n">
         <v>162177.170399998</v>
       </c>
-      <c r="E17" s="21" t="n">
+      <c r="E17" s="26" t="n">
         <v>826</v>
       </c>
-      <c r="F17" s="22" t="n">
+      <c r="F17" s="27" t="n">
         <f aca="false">D17-B17</f>
-        <v>45158.2919999979</v>
-      </c>
+        <v>45158.291999998</v>
+      </c>
+      <c r="G17" s="0"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="20" t="n">
+      <c r="B18" s="25" t="n">
         <v>192347.280000001</v>
       </c>
-      <c r="C18" s="21" t="n">
+      <c r="C18" s="26" t="n">
         <v>311</v>
       </c>
-      <c r="D18" s="20" t="n">
+      <c r="D18" s="25" t="n">
         <v>371087.999999999</v>
       </c>
-      <c r="E18" s="21" t="n">
+      <c r="E18" s="26" t="n">
         <v>600</v>
       </c>
-      <c r="F18" s="22" t="n">
+      <c r="F18" s="27" t="n">
         <f aca="false">D18-B18</f>
         <v>178740.719999998</v>
       </c>
+      <c r="G18" s="0"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="24" t="s">
+      <c r="A19" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="25" t="n">
-        <v>395133.859799999</v>
-      </c>
-      <c r="C19" s="26" t="n">
+      <c r="B19" s="31" t="n">
+        <v>395133.859799998</v>
+      </c>
+      <c r="C19" s="32" t="n">
         <v>438</v>
       </c>
-      <c r="D19" s="25" t="n">
-        <v>717195.019499995</v>
-      </c>
-      <c r="E19" s="26" t="n">
+      <c r="D19" s="31" t="n">
+        <v>717195.019499994</v>
+      </c>
+      <c r="E19" s="32" t="n">
         <v>795</v>
       </c>
-      <c r="F19" s="27" t="n">
+      <c r="F19" s="33" t="n">
         <f aca="false">D19-B19</f>
         <v>322061.159699996</v>
       </c>
+      <c r="G19" s="0"/>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0"/>
+      <c r="B20" s="0"/>
+      <c r="C20" s="0"/>
+      <c r="D20" s="0"/>
+      <c r="E20" s="0"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="0"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F7:F19">
+  <conditionalFormatting sqref="F6:F19">
     <cfRule type="cellIs" priority="2" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>-10000</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="between" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>-10000</formula>
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3677,242 +3894,243 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="9.92"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="9.92"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="34" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="6" t="s">
+      <c r="B1" s="35"/>
+      <c r="C1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="30"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="32" t="n">
+      <c r="C2" s="38" t="n">
         <v>2021</v>
       </c>
-      <c r="D2" s="33" t="n">
+      <c r="D2" s="39" t="n">
         <v>2022</v>
       </c>
-      <c r="E2" s="14" t="s">
-        <v>35</v>
+      <c r="E2" s="19" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="34" t="s">
+      <c r="A3" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="35" t="n">
+      <c r="C3" s="21" t="n">
         <v>492422.616400001</v>
       </c>
-      <c r="D3" s="36" t="n">
+      <c r="D3" s="41" t="n">
         <v>201445.6158</v>
       </c>
-      <c r="E3" s="18" t="n">
+      <c r="E3" s="23" t="n">
         <f aca="false">D3-C3</f>
-        <v>-290977.0006</v>
+        <v>-290977.000600001</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="37"/>
-      <c r="B4" s="24" t="s">
+      <c r="A4" s="42"/>
+      <c r="B4" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="38" t="n">
+      <c r="C4" s="31" t="n">
         <v>290100.266199999</v>
       </c>
-      <c r="D4" s="39" t="n">
+      <c r="D4" s="43" t="n">
         <v>54235.3581</v>
       </c>
-      <c r="E4" s="22" t="n">
+      <c r="E4" s="27" t="n">
         <f aca="false">D4-C4</f>
         <v>-235864.908099999</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="34" t="s">
+      <c r="A5" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="35" t="n">
+      <c r="C5" s="21" t="n">
         <v>798965.10539999</v>
       </c>
-      <c r="D5" s="36" t="n">
+      <c r="D5" s="41" t="n">
         <v>682940.656799996</v>
       </c>
-      <c r="E5" s="22" t="n">
+      <c r="E5" s="27" t="n">
         <f aca="false">D5-C5</f>
         <v>-116024.448599994</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="37"/>
-      <c r="B6" s="24" t="s">
+      <c r="A6" s="42"/>
+      <c r="B6" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="38" t="n">
+      <c r="C6" s="31" t="n">
         <v>771433.033300014</v>
       </c>
-      <c r="D6" s="39" t="n">
+      <c r="D6" s="43" t="n">
         <v>683705.172900009</v>
       </c>
-      <c r="E6" s="22" t="n">
+      <c r="E6" s="27" t="n">
         <f aca="false">D6-C6</f>
-        <v>-87727.8604000052</v>
+        <v>-87727.860400005</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="37"/>
-      <c r="B7" s="24" t="s">
+      <c r="A7" s="42"/>
+      <c r="B7" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="38" t="n">
+      <c r="C7" s="31" t="n">
         <v>48611.823</v>
       </c>
-      <c r="D7" s="40"/>
-      <c r="E7" s="22" t="n">
+      <c r="D7" s="44"/>
+      <c r="E7" s="27" t="n">
         <f aca="false">D7-C7</f>
         <v>-48611.823</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="34" t="s">
+      <c r="A8" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="35" t="n">
+      <c r="C8" s="21" t="n">
         <v>46610.1597</v>
       </c>
-      <c r="D8" s="41"/>
-      <c r="E8" s="22" t="n">
+      <c r="D8" s="45"/>
+      <c r="E8" s="27" t="n">
         <f aca="false">D8-C8</f>
         <v>-46610.1597</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="42" t="s">
+      <c r="A9" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="43" t="s">
+      <c r="B9" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="44" t="n">
+      <c r="C9" s="48" t="n">
         <v>242005.227899996</v>
       </c>
-      <c r="D9" s="45" t="n">
+      <c r="D9" s="49" t="n">
         <v>237267.768299996</v>
       </c>
-      <c r="E9" s="22" t="n">
+      <c r="E9" s="27" t="n">
         <f aca="false">D9-C9</f>
-        <v>-4737.45959999983</v>
+        <v>-4737.4596</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="42" t="s">
+      <c r="A10" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="43" t="s">
+      <c r="B10" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="44" t="n">
+      <c r="C10" s="48" t="n">
         <v>11745.012</v>
       </c>
-      <c r="D10" s="45" t="n">
+      <c r="D10" s="49" t="n">
         <v>11545.944</v>
       </c>
-      <c r="E10" s="22" t="n">
+      <c r="E10" s="27" t="n">
         <f aca="false">D10-C10</f>
-        <v>-199.067999999999</v>
+        <v>-199.068000000001</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="42" t="s">
+      <c r="A11" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="43" t="s">
+      <c r="B11" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="44" t="n">
+      <c r="C11" s="48" t="n">
         <v>10141.2</v>
       </c>
-      <c r="D11" s="45" t="n">
+      <c r="D11" s="49" t="n">
         <v>12545.04</v>
       </c>
-      <c r="E11" s="22" t="n">
+      <c r="E11" s="27" t="n">
         <f aca="false">D11-C11</f>
-        <v>2403.84000000003</v>
+        <v>2403.84</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="37"/>
-      <c r="B12" s="24" t="s">
+      <c r="A12" s="42"/>
+      <c r="B12" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="38" t="n">
+      <c r="C12" s="31" t="n">
         <v>23879.8053</v>
       </c>
-      <c r="D12" s="39" t="n">
+      <c r="D12" s="43" t="n">
         <v>33893.9171999999</v>
       </c>
-      <c r="E12" s="22" t="n">
+      <c r="E12" s="27" t="n">
         <f aca="false">D12-C12</f>
-        <v>10014.1119</v>
+        <v>10014.1118999999</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="34" t="s">
+      <c r="A13" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="35" t="n">
+      <c r="C13" s="21" t="n">
         <v>24295.6197</v>
       </c>
-      <c r="D13" s="36" t="n">
+      <c r="D13" s="41" t="n">
         <v>36566.1347</v>
       </c>
-      <c r="E13" s="22" t="n">
+      <c r="E13" s="27" t="n">
         <f aca="false">D13-C13</f>
         <v>12270.515</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="46" t="s">
+      <c r="A14" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="47" t="s">
+      <c r="B14" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="48" t="n">
+      <c r="C14" s="21" t="n">
         <v>31742.2876</v>
       </c>
-      <c r="D14" s="49" t="n">
+      <c r="D14" s="41" t="n">
         <v>45225.7372000001</v>
       </c>
-      <c r="E14" s="22" t="n">
+      <c r="E14" s="27" t="n">
         <f aca="false">D14-C14</f>
         <v>13483.4496000001</v>
       </c>
@@ -3928,116 +4146,123 @@
       <c r="D15" s="53" t="n">
         <v>43540.3060000001</v>
       </c>
-      <c r="E15" s="22" t="n">
+      <c r="E15" s="27" t="n">
         <f aca="false">D15-C15</f>
         <v>15168.8808000001</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="42" t="s">
+      <c r="A16" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="43" t="s">
+      <c r="B16" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="44" t="n">
+      <c r="C16" s="48" t="n">
         <v>73092.1728000002</v>
       </c>
-      <c r="D16" s="45" t="n">
+      <c r="D16" s="49" t="n">
         <v>92859.2384000003</v>
       </c>
-      <c r="E16" s="22" t="n">
+      <c r="E16" s="27" t="n">
         <f aca="false">D16-C16</f>
         <v>19767.0656000001</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="42" t="s">
+      <c r="A17" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="43" t="s">
+      <c r="B17" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="44" t="n">
+      <c r="C17" s="48" t="n">
         <v>70991.4548000001</v>
       </c>
-      <c r="D17" s="45" t="n">
+      <c r="D17" s="49" t="n">
         <v>115404.827999999</v>
       </c>
-      <c r="E17" s="22" t="n">
+      <c r="E17" s="27" t="n">
         <f aca="false">D17-C17</f>
-        <v>44413.3731999994</v>
+        <v>44413.3731999989</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="42" t="s">
+      <c r="A18" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="43" t="s">
+      <c r="B18" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="44" t="n">
+      <c r="C18" s="48" t="n">
         <v>117018.8784</v>
       </c>
-      <c r="D18" s="45" t="n">
+      <c r="D18" s="49" t="n">
         <v>162177.170399998</v>
       </c>
-      <c r="E18" s="22" t="n">
+      <c r="E18" s="27" t="n">
         <f aca="false">D18-C18</f>
-        <v>45158.2919999979</v>
+        <v>45158.291999998</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="37"/>
-      <c r="B19" s="24" t="s">
+      <c r="A19" s="42"/>
+      <c r="B19" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="C19" s="38" t="n">
+      <c r="C19" s="31" t="n">
         <v>193056.269399999</v>
       </c>
-      <c r="D19" s="39" t="n">
+      <c r="D19" s="43" t="n">
         <v>352733.651099997</v>
       </c>
-      <c r="E19" s="22" t="n">
+      <c r="E19" s="27" t="n">
         <f aca="false">D19-C19</f>
         <v>159677.381699998</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="34" t="s">
+      <c r="A20" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="15" t="s">
+      <c r="B20" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="C20" s="35" t="n">
+      <c r="C20" s="21" t="n">
         <v>202077.590399999</v>
       </c>
-      <c r="D20" s="36" t="n">
+      <c r="D20" s="41" t="n">
         <v>364461.368399997</v>
       </c>
-      <c r="E20" s="22" t="n">
+      <c r="E20" s="27" t="n">
         <f aca="false">D20-C20</f>
         <v>162383.777999998</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="42" t="s">
+      <c r="A21" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="43" t="s">
+      <c r="B21" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="C21" s="44" t="n">
+      <c r="C21" s="48" t="n">
         <v>192347.280000001</v>
       </c>
-      <c r="D21" s="45" t="n">
+      <c r="D21" s="49" t="n">
         <v>371087.999999999</v>
       </c>
-      <c r="E21" s="27" t="n">
+      <c r="E21" s="33" t="n">
         <f aca="false">D21-C21</f>
         <v>178740.719999998</v>
       </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0"/>
+      <c r="B22" s="0"/>
+      <c r="C22" s="0"/>
+      <c r="D22" s="0"/>
+      <c r="E22" s="6"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E21">

</xml_diff>